<commit_message>
41 Elizabeth Ct package r9: marketing example, map previews, calculator copy
Adds section 4 with the 82 Spring Lane example, pin-anchored comp previews
and a subject marker on the map, a consistent spacing scale, the package
calculator with plain-language fee wording, and a refreshed PDF and net sheet.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/p/41-elizabeth-ct-4b5cd4/41-elizabeth-ct-seller-net-proceeds.xlsx
+++ b/p/41-elizabeth-ct-4b5cd4/41-elizabeth-ct-seller-net-proceeds.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Net Proceeds" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Net Proceeds'!$A$1:$D$21</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Net Proceeds'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +31,7 @@
     <t xml:space="preserve">41 Elizabeth Ct, Secaucus, NJ 07094</t>
   </si>
   <si>
-    <t xml:space="preserve">Michael Gonnelli | The Gonnelli Group | RE/MAX Select | 201-240-8422</t>
+    <t xml:space="preserve">Michael Gonnelli | The Gonnelli Group at RE/MAX Select | 201-240-8422 | michael@thegonnelligroup.com</t>
   </si>
   <si>
     <t xml:space="preserve">Compensation rate</t>
@@ -79,7 +79,7 @@
     <t xml:space="preserve">Payoff status</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue cells are editable. Leave mortgage payoff as Not provided until known; enter 0 only if confirmed. Other liens, prorations and unlisted costs are excluded unless entered in Other costs. Reduced RTF requires confirmed eligibility with your attorney. Estimates only, not a closing statement. NJ RTF and July 2025 Graduated Percent Fee schedules apply.</t>
+    <t xml:space="preserve">Blue cells are editable. Leave mortgage payoff as Not provided until known; enter 0 only if confirmed. Other liens, prorations and unlisted costs are excluded unless entered in Other costs. B6 NO uses standard RTF; YES uses the partial exemption for eligible senior, blind or disabled owner-occupants. Confirm all NJ RTF-1 residency and ownership conditions with your attorney first. Veteran status alone does not qualify; annual property-tax benefits and full RTF exemptions are separate. Conditions: https://www.nj.gov/treasury/taxation/pdf/other_forms/lpt/rtfexempt.pdf. Estimates only. NJ RTF and July 2025 Graduated Percent Fee schedules apply.</t>
   </si>
 </sst>
 </file>
@@ -186,6 +186,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -211,10 +215,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -302,8 +302,8 @@
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>1504440</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>27000</xdr:rowOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>628200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -513,14 +513,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="22"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -530,16 +530,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>0.04</v>
       </c>
     </row>
@@ -547,7 +550,7 @@
       <c r="A6" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
     </row>
@@ -555,13 +558,13 @@
       <c r="A8" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <v>750000</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="5" t="n">
         <v>775000</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <v>800000</v>
       </c>
     </row>
@@ -569,15 +572,15 @@
       <c r="A9" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <f aca="false">ROUND(IF(ROUND(B8,2)&lt;=350000,IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(B8,2),150000)-0)/500,0)*0.5+ROUNDUP(MAX(0,MIN(ROUND(B8,2),350000)-150000)/500,0)*1.25,ROUNDUP(MAX(0,MIN(ROUND(B8,2),150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(ROUND(B8,2),200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(ROUND(B8,2),350000)-200000)/500,0)*3.9),IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(B8,2),150000)-0)/500,0)*1.4+ROUNDUP(MAX(0,MIN(ROUND(B8,2),550000)-150000)/500,0)*2.15+ROUNDUP(MAX(0,MIN(ROUND(B8,2),850000)-550000)/500,0)*2.65+ROUNDUP(MAX(0,MIN(ROUND(B8,2),1000000)-850000)/500,0)*3.15+ROUNDUP(MAX(0,ROUND(B8,2)-1000000)/500,0)*3.4,ROUNDUP(MAX(0,MIN(ROUND(B8,2),150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(ROUND(B8,2),200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(ROUND(B8,2),550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(ROUND(B8,2),850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(ROUND(B8,2),1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,ROUND(B8,2)-1000000)/500,0)*6.05)),2)</f>
         <v>6775</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="6" t="n">
         <f aca="false">ROUND(IF(ROUND(C8,2)&lt;=350000,IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(C8,2),150000)-0)/500,0)*0.5+ROUNDUP(MAX(0,MIN(ROUND(C8,2),350000)-150000)/500,0)*1.25,ROUNDUP(MAX(0,MIN(ROUND(C8,2),150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(ROUND(C8,2),200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(ROUND(C8,2),350000)-200000)/500,0)*3.9),IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(C8,2),150000)-0)/500,0)*1.4+ROUNDUP(MAX(0,MIN(ROUND(C8,2),550000)-150000)/500,0)*2.15+ROUNDUP(MAX(0,MIN(ROUND(C8,2),850000)-550000)/500,0)*2.65+ROUNDUP(MAX(0,MIN(ROUND(C8,2),1000000)-850000)/500,0)*3.15+ROUNDUP(MAX(0,ROUND(C8,2)-1000000)/500,0)*3.4,ROUNDUP(MAX(0,MIN(ROUND(C8,2),150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(ROUND(C8,2),200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(ROUND(C8,2),550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(ROUND(C8,2),850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(ROUND(C8,2),1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,ROUND(C8,2)-1000000)/500,0)*6.05)),2)</f>
         <v>7040</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="6" t="n">
         <f aca="false">ROUND(IF(ROUND(D8,2)&lt;=350000,IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*0.5+ROUNDUP(MAX(0,MIN(ROUND(D8,2),350000)-150000)/500,0)*1.25,ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(ROUND(D8,2),200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(ROUND(D8,2),350000)-200000)/500,0)*3.9),IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*1.4+ROUNDUP(MAX(0,MIN(ROUND(D8,2),550000)-150000)/500,0)*2.15+ROUNDUP(MAX(0,MIN(ROUND(D8,2),850000)-550000)/500,0)*2.65+ROUNDUP(MAX(0,MIN(ROUND(D8,2),1000000)-850000)/500,0)*3.15+ROUNDUP(MAX(0,ROUND(D8,2)-1000000)/500,0)*3.4,ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(ROUND(D8,2),200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(ROUND(D8,2),550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(ROUND(D8,2),850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(ROUND(D8,2),1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,ROUND(D8,2)-1000000)/500,0)*6.05)),2)</f>
         <v>7305</v>
       </c>
@@ -586,15 +589,15 @@
       <c r="A10" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <f aca="false">ROUND(ROUND(B8,2)*IF(ROUND(B8,2)&lt;=1000000,0,IF(ROUND(B8,2)&lt;=2000000,0.01,IF(ROUND(B8,2)&lt;=2500000,0.02,IF(ROUND(B8,2)&lt;=3000000,0.025,IF(ROUND(B8,2)&lt;=3500000,0.03,0.035))))),2)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6" t="n">
         <f aca="false">ROUND(ROUND(C8,2)*IF(ROUND(C8,2)&lt;=1000000,0,IF(ROUND(C8,2)&lt;=2000000,0.01,IF(ROUND(C8,2)&lt;=2500000,0.02,IF(ROUND(C8,2)&lt;=3000000,0.025,IF(ROUND(C8,2)&lt;=3500000,0.03,0.035))))),2)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="6" t="n">
         <f aca="false">ROUND(ROUND(D8,2)*IF(ROUND(D8,2)&lt;=1000000,0,IF(ROUND(D8,2)&lt;=2000000,0.01,IF(ROUND(D8,2)&lt;=2500000,0.02,IF(ROUND(D8,2)&lt;=3000000,0.025,IF(ROUND(D8,2)&lt;=3500000,0.03,0.035))))),2)</f>
         <v>0</v>
       </c>
@@ -603,15 +606,15 @@
       <c r="A11" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="6" t="n">
         <f aca="false">ROUND($B$5*ROUND(B8,2),2)</f>
         <v>30000</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="6" t="n">
         <f aca="false">ROUND($B$5*ROUND(C8,2),2)</f>
         <v>31000</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="6" t="n">
         <f aca="false">ROUND($B$5*ROUND(D8,2),2)</f>
         <v>32000</v>
       </c>
@@ -620,13 +623,13 @@
       <c r="A12" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="5" t="n">
         <v>1500</v>
       </c>
     </row>
@@ -634,13 +637,13 @@
       <c r="A13" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>200</v>
       </c>
     </row>
@@ -648,29 +651,29 @@
       <c r="A14" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="6" t="n">
         <f aca="false">ROUND(ROUND(B8,2)-SUM(B9:B11)-ROUND(B12,2)-ROUND(B13,2)-ROUND(B14,2),2)</f>
         <v>711525</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="6" t="n">
         <f aca="false">ROUND(ROUND(C8,2)-SUM(C9:C11)-ROUND(C12,2)-ROUND(C13,2)-ROUND(C14,2),2)</f>
         <v>735260</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="6" t="n">
         <f aca="false">ROUND(ROUND(D8,2)-SUM(D9:D11)-ROUND(D12,2)-ROUND(D13,2)-ROUND(D14,2),2)</f>
         <v>758995</v>
       </c>
@@ -679,29 +682,29 @@
       <c r="A16" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="6" t="n">
         <f aca="false">ROUND(B15-IF(ISNUMBER(B16),ROUND(B16,2),0),2)</f>
         <v>711525</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="6" t="n">
         <f aca="false">ROUND(C15-IF(ISNUMBER(C16),ROUND(C16,2),0),2)</f>
         <v>735260</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="6" t="n">
         <f aca="false">ROUND(D15-IF(ISNUMBER(D16),ROUND(D16,2),0),2)</f>
         <v>758995</v>
       </c>
@@ -710,42 +713,55 @@
       <c r="A18" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="8" t="str">
+      <c r="B18" s="9" t="str">
         <f aca="false">IF(ISNUMBER(B16),"After entered payoff","Before payoff (not provided)")</f>
         <v>Before payoff (not provided)</v>
       </c>
-      <c r="C18" s="8" t="str">
+      <c r="C18" s="9" t="str">
         <f aca="false">IF(ISNUMBER(C16),"After entered payoff","Before payoff (not provided)")</f>
         <v>Before payoff (not provided)</v>
       </c>
-      <c r="D18" s="8" t="str">
+      <c r="D18" s="9" t="str">
         <f aca="false">IF(ISNUMBER(D16),"After entered payoff","Before payoff (not provided)")</f>
         <v>Before payoff (not provided)</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A19:D21"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A19:D23"/>
   </mergeCells>
   <dataValidations count="9">
     <dataValidation allowBlank="false" error="Enter a nonnegative amount." errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B12:D14" type="decimal">

</xml_diff>